<commit_message>
add follow-up fields to import/export and include first_positive_lab in canned exports
</commit_message>
<xml_diff>
--- a/test/fixtures/files/Sara-Alert-Format-Exposure-Workflow.xlsx
+++ b/test/fixtures/files/Sara-Alert-Format-Exposure-Workflow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twong/Documents/SARA-ALERT/SaraAlert/test/fixtures/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C885723B-7DF2-E748-80C7-6A6445D63090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF7CD85-5FB5-3847-B3AC-B2ECAE229887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10120" yWindow="2140" windowWidth="21640" windowHeight="14440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monitorees" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="478">
   <si>
     <t>First Name</t>
   </si>
@@ -1439,6 +1439,21 @@
   </si>
   <si>
     <t>pfizerbiontech covid19 vaccine</t>
+  </si>
+  <si>
+    <t>Follow-Up Reason</t>
+  </si>
+  <si>
+    <t>Follow-Up Note</t>
+  </si>
+  <si>
+    <t>Duplicate</t>
+  </si>
+  <si>
+    <t>Hospitalized</t>
+  </si>
+  <si>
+    <t>example note</t>
   </si>
 </sst>
 </file>
@@ -1791,7 +1806,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DH12"/>
+  <dimension ref="A1:DJ12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -1906,9 +1921,11 @@
     <col min="110" max="110" width="25.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="111" max="111" width="21.1640625" bestFit="1" customWidth="1"/>
     <col min="112" max="112" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2245,8 +2262,14 @@
       <c r="DH1" t="s">
         <v>455</v>
       </c>
+      <c r="DI1" t="s">
+        <v>473</v>
+      </c>
+      <c r="DJ1" t="s">
+        <v>474</v>
+      </c>
     </row>
-    <row r="2" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -2556,8 +2579,14 @@
       <c r="DH2" t="s">
         <v>462</v>
       </c>
+      <c r="DI2" t="s">
+        <v>475</v>
+      </c>
+      <c r="DJ2" t="s">
+        <v>477</v>
+      </c>
     </row>
-    <row r="3" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>118</v>
       </c>
@@ -2861,8 +2890,11 @@
       <c r="DG3">
         <v>2</v>
       </c>
+      <c r="DI3" t="s">
+        <v>476</v>
+      </c>
     </row>
-    <row r="4" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>142</v>
       </c>
@@ -3167,7 +3199,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>163</v>
       </c>
@@ -3415,7 +3447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
         <v>176</v>
       </c>
@@ -3681,7 +3713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
         <v>197</v>
       </c>
@@ -3950,7 +3982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
         <v>216</v>
       </c>
@@ -4207,7 +4239,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
         <v>235</v>
       </c>
@@ -4488,7 +4520,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="10" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
         <v>251</v>
       </c>
@@ -4769,7 +4801,7 @@
         <v>9999</v>
       </c>
     </row>
-    <row r="11" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
         <v>271</v>
       </c>
@@ -5026,7 +5058,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="12" spans="1:112" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
         <v>293</v>
       </c>

</xml_diff>